<commit_message>
Öffentliche Recon-/PII-Daten bereinigen und Fixed-Fee-Calculator umbenennen.
Excel-Templates ohne echte Patienten-/Labornamen, Deploy-Pfad als Secret,
ADR entschärft; WaelFixedFeeCalculator → FixedFeeIncomeCalculator
(weiterhin dynamisch über commission_type, nicht an Code WA gebunden).
</commit_message>
<xml_diff>
--- a/resources/templates/drs_income_template.xlsx
+++ b/resources/templates/drs_income_template.xlsx
@@ -164,14 +164,14 @@
         <sz val="11"/>
         <u val="none"/>
       </rPr>
-      <t xml:space="preserve"> Wael </t>
+      <t xml:space="preserve"> Doctor C </t>
     </r>
   </si>
   <si>
     <t>2021-May</t>
   </si>
   <si>
-    <t>Dr Wael (Surg)</t>
+    <t>Doctor C (Surg)</t>
   </si>
   <si>
     <t>Date</t>
@@ -336,43 +336,43 @@
     <t>Item</t>
   </si>
   <si>
-    <t>MIDDLE EAST LAB</t>
+    <t>Lab Vendor 1</t>
   </si>
   <si>
-    <t>Qualia</t>
+    <t>Lab Vendor 2</t>
   </si>
   <si>
-    <t>AL MAHA</t>
+    <t>Lab Vendor 3</t>
   </si>
   <si>
-    <t xml:space="preserve">pearl lab </t>
+    <t xml:space="preserve">Lab Vendor 4</t>
   </si>
   <si>
-    <t>Oral Design</t>
+    <t>Lab Vendor 5</t>
   </si>
   <si>
-    <t>Sahara Lab</t>
+    <t>Lab Vendor 6</t>
   </si>
   <si>
-    <t>Italian Lab</t>
+    <t>Lab Vendor 7</t>
   </si>
   <si>
-    <t>Diamond Lab</t>
+    <t>Lab Vendor 8</t>
   </si>
   <si>
     <t>Dr. Lab cost</t>
   </si>
   <si>
-    <t>Dr.Anas</t>
+    <t>Doctor A</t>
   </si>
   <si>
     <t>Dr.Riyadh</t>
   </si>
   <si>
-    <t>Dr.Irina</t>
+    <t>Doctor B</t>
   </si>
   <si>
-    <t>Dr.WAEL</t>
+    <t>Doctor C</t>
   </si>
   <si>
     <t>Column5</t>
@@ -1124,10 +1124,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve" id="1" name="Table1" displayName="Table_1" ref="N2:T13" headerRowCount="1" totalsRowCount="0">
   <tableColumns count="7">
     <tableColumn id="1" name="Dr. Lab cost"/>
-    <tableColumn id="2" name="Dr.Anas"/>
+    <tableColumn id="2" name="Doctor A"/>
     <tableColumn id="3" name="Dr.Riyadh"/>
-    <tableColumn id="4" name="Dr.Irina"/>
-    <tableColumn id="5" name="Dr.WAEL"/>
+    <tableColumn id="4" name="Doctor B"/>
+    <tableColumn id="5" name="Doctor C"/>
     <tableColumn id="6" name="Column5"/>
     <tableColumn id="7" name="Column6"/>
   </tableColumns>

</xml_diff>